<commit_message>
feat: Integracion Zoho Mail REST API, nuevo rol Contabilidad - Caja Chica, catalogo unificado de proveedores y selector avanzado de aprobadores
</commit_message>
<xml_diff>
--- a/LISTA_USUARIOS.xlsx
+++ b/LISTA_USUARIOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\franco\Desktop\sistema_solicitud\New folder\sistema_solicitud\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E7006F4-8C49-4A01-AC49-5E65A9554BEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CE5F563-6D30-44B5-B963-F692F7065D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9300" yWindow="1755" windowWidth="12915" windowHeight="11055" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -836,7 +836,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -848,6 +848,14 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -922,10 +930,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -939,6 +948,7 @@
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -949,7 +959,8 @@
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1298,14 +1309,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="9"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="10"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1934,7 +1945,7 @@
       <c r="B33" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="C33" s="2" t="s">
+      <c r="C33" s="7" t="s">
         <v>147</v>
       </c>
       <c r="D33" s="4" t="s">
@@ -2241,7 +2252,7 @@
         <v>215</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>217</v>
+        <v>267</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>255</v>
@@ -2288,14 +2299,14 @@
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" s="7" t="s">
+      <c r="A51" s="8" t="s">
         <v>210</v>
       </c>
-      <c r="B51" s="8"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="9"/>
+      <c r="B51" s="9"/>
+      <c r="C51" s="9"/>
+      <c r="D51" s="9"/>
+      <c r="E51" s="9"/>
+      <c r="F51" s="10"/>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="2" t="s">
@@ -2364,7 +2375,7 @@
       <c r="B55" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C55" s="2" t="s">
+      <c r="C55" s="7" t="s">
         <v>168</v>
       </c>
       <c r="D55" s="4" t="s">
@@ -2658,14 +2669,14 @@
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A70" s="7" t="s">
+      <c r="A70" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="B70" s="8"/>
-      <c r="C70" s="8"/>
-      <c r="D70" s="8"/>
-      <c r="E70" s="8"/>
-      <c r="F70" s="9"/>
+      <c r="B70" s="9"/>
+      <c r="C70" s="9"/>
+      <c r="D70" s="9"/>
+      <c r="E70" s="9"/>
+      <c r="F70" s="10"/>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
@@ -2814,14 +2825,14 @@
       <c r="B78" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="C78" s="7" t="s">
         <v>190</v>
       </c>
       <c r="D78" s="4" t="s">
         <v>215</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>217</v>
+        <v>267</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>261</v>
@@ -3054,7 +3065,7 @@
       <c r="B90" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="C90" s="7" t="s">
         <v>201</v>
       </c>
       <c r="D90" s="4" t="s">
@@ -3194,6 +3205,12 @@
     <mergeCell ref="A70:F70"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C33" r:id="rId1" xr:uid="{330E161C-A54C-4A83-9BC8-3B87D118ACB0}"/>
+    <hyperlink ref="C55" r:id="rId2" xr:uid="{E7298ADC-5B79-43C7-81DC-031BC7146A41}"/>
+    <hyperlink ref="C78" r:id="rId3" xr:uid="{FE2A8D02-FA74-4181-8372-15178926B95C}"/>
+    <hyperlink ref="C90" r:id="rId4" xr:uid="{D0538DA9-A632-47DA-9B71-3DDD76331E2B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>